<commit_message>
updating prediction and offset file
</commit_message>
<xml_diff>
--- a/data/raw/f1_circuits_2018_2026_extended.xlsx
+++ b/data/raw/f1_circuits_2018_2026_extended.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gandj\Documents\F1\Manual\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{560BC67E-75B2-4C55-A241-1CEE4B5F1262}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F298854-7142-4614-8EA0-44FCCFFDA890}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3120" yWindow="3120" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Circuits 2018-2026" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="575" uniqueCount="245">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="575" uniqueCount="243">
   <si>
     <t>Circuit</t>
   </si>
@@ -544,21 +544,12 @@
     <t>Barajas</t>
   </si>
   <si>
-    <t>5.474 km</t>
-  </si>
-  <si>
     <t>22</t>
   </si>
   <si>
     <t>2026</t>
   </si>
   <si>
-    <t>Mixed / provisional</t>
-  </si>
-  <si>
-    <t>Low</t>
-  </si>
-  <si>
     <t>Marina Bay Street Circuit</t>
   </si>
   <si>
@@ -761,6 +752,9 @@
   </si>
   <si>
     <t>Madrid Grand Prix</t>
+  </si>
+  <si>
+    <t>5.416 km</t>
   </si>
 </sst>
 </file>
@@ -1038,43 +1032,43 @@
         <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>240</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="L1" s="1" t="s">
         <v>233</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>234</v>
       </c>
-      <c r="J1" s="1" t="s">
-        <v>243</v>
-      </c>
-      <c r="K1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>236</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>237</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>238</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>239</v>
       </c>
       <c r="P1" s="1" t="s">
         <v>6</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="S1" s="1" t="s">
         <v>8</v>
@@ -2602,40 +2596,40 @@
         <v>118</v>
       </c>
       <c r="F24" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="G24" s="2" t="s">
         <v>172</v>
       </c>
-      <c r="G24" s="2" t="s">
+      <c r="H24" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="I24" s="2" t="s">
         <v>173</v>
-      </c>
-      <c r="H24" s="2" t="s">
-        <v>244</v>
-      </c>
-      <c r="I24" s="2" t="s">
-        <v>174</v>
       </c>
       <c r="J24" s="2" t="s">
         <v>54</v>
       </c>
       <c r="K24" s="2" t="s">
-        <v>175</v>
+        <v>87</v>
       </c>
       <c r="L24" s="4">
-        <v>900</v>
+        <v>1300</v>
       </c>
       <c r="M24" s="2">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="N24" s="2">
+        <v>6</v>
+      </c>
+      <c r="O24" s="2">
         <v>8</v>
       </c>
-      <c r="O24" s="2">
-        <v>4</v>
-      </c>
       <c r="P24" s="2" t="s">
-        <v>176</v>
+        <v>23</v>
       </c>
       <c r="Q24" s="3">
-        <v>4.0199999999999996</v>
+        <v>4.0599999999999996</v>
       </c>
       <c r="R24" s="2" t="s">
         <v>48</v>
@@ -2655,7 +2649,7 @@
     </row>
     <row r="25" spans="1:22" ht="15" customHeight="1">
       <c r="A25" s="2" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="B25" s="2" t="s">
         <v>13</v>
@@ -2664,19 +2658,19 @@
         <v>39</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="G25" s="2" t="s">
         <v>43</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="I25" s="2" t="s">
         <v>20</v>
@@ -2723,7 +2717,7 @@
     </row>
     <row r="26" spans="1:22" ht="15" customHeight="1">
       <c r="A26" s="2" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="B26" s="2" t="s">
         <v>13</v>
@@ -2732,7 +2726,7 @@
         <v>39</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>134</v>
@@ -2744,16 +2738,16 @@
         <v>43</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="I26" s="2" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="J26" s="2" t="s">
         <v>46</v>
       </c>
       <c r="K26" s="2" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="L26" s="4">
         <v>1310</v>
@@ -2791,7 +2785,7 @@
     </row>
     <row r="27" spans="1:22" ht="15" customHeight="1">
       <c r="A27" s="2" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="B27" s="2" t="s">
         <v>30</v>
@@ -2800,19 +2794,19 @@
         <v>14</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="E27" s="2" t="s">
         <v>139</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="G27" s="2" t="s">
         <v>34</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="I27" s="2" t="s">
         <v>53</v>
@@ -2859,7 +2853,7 @@
     </row>
     <row r="28" spans="1:22" ht="15" customHeight="1">
       <c r="A28" s="2" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="B28" s="2" t="s">
         <v>30</v>
@@ -2868,19 +2862,19 @@
         <v>14</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="G28" s="2" t="s">
         <v>86</v>
       </c>
       <c r="H28" s="2" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="I28" s="2" t="s">
         <v>71</v>
@@ -2927,7 +2921,7 @@
     </row>
     <row r="29" spans="1:22" ht="15" customHeight="1">
       <c r="A29" s="2" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>30</v>
@@ -2936,22 +2930,22 @@
         <v>14</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="G29" s="2" t="s">
         <v>18</v>
       </c>
       <c r="H29" s="2" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="I29" s="2" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="J29" s="2" t="s">
         <v>46</v>
@@ -2995,7 +2989,7 @@
     </row>
     <row r="30" spans="1:22" ht="15" customHeight="1">
       <c r="A30" s="2" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="B30" s="2" t="s">
         <v>30</v>
@@ -3004,19 +2998,19 @@
         <v>14</v>
       </c>
       <c r="D30" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="F30" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="G30" s="2" t="s">
         <v>203</v>
       </c>
-      <c r="E30" s="2" t="s">
+      <c r="H30" s="2" t="s">
         <v>204</v>
-      </c>
-      <c r="F30" s="2" t="s">
-        <v>205</v>
-      </c>
-      <c r="G30" s="2" t="s">
-        <v>206</v>
-      </c>
-      <c r="H30" s="2" t="s">
-        <v>207</v>
       </c>
       <c r="I30" s="2" t="s">
         <v>71</v>
@@ -3063,7 +3057,7 @@
     </row>
     <row r="31" spans="1:22" ht="15" customHeight="1">
       <c r="A31" s="2" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="B31" s="2" t="s">
         <v>30</v>
@@ -3072,22 +3066,22 @@
         <v>14</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="G31" s="2" t="s">
         <v>34</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="I31" s="2" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="J31" s="2" t="s">
         <v>108</v>
@@ -3131,28 +3125,28 @@
     </row>
     <row r="32" spans="1:22" ht="15" customHeight="1">
       <c r="A32" s="2" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="B32" s="2" t="s">
         <v>30</v>
       </c>
       <c r="C32" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="F32" s="2" t="s">
         <v>215</v>
       </c>
-      <c r="D32" s="2" t="s">
+      <c r="G32" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="H32" s="2" t="s">
         <v>216</v>
-      </c>
-      <c r="E32" s="2" t="s">
-        <v>217</v>
-      </c>
-      <c r="F32" s="2" t="s">
-        <v>218</v>
-      </c>
-      <c r="G32" s="2" t="s">
-        <v>206</v>
-      </c>
-      <c r="H32" s="2" t="s">
-        <v>219</v>
       </c>
       <c r="I32" s="2" t="s">
         <v>20</v>
@@ -3199,7 +3193,7 @@
     </row>
     <row r="33" spans="1:22" ht="15" customHeight="1">
       <c r="A33" s="2" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="B33" s="2" t="s">
         <v>30</v>
@@ -3208,19 +3202,19 @@
         <v>39</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="G33" s="2" t="s">
         <v>18</v>
       </c>
       <c r="H33" s="2" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="I33" s="2" t="s">
         <v>71</v>
@@ -3281,32 +3275,32 @@
   <sheetData>
     <row r="1" spans="1:2" ht="15.95" customHeight="1">
       <c r="A1" s="5" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="B1" s="5"/>
     </row>
     <row r="2" spans="1:2" ht="15" customHeight="1">
       <c r="A2" s="6" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="15" customHeight="1">
       <c r="A3" s="6" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="15" customHeight="1">
       <c r="A4" s="6" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="15" customHeight="1">
@@ -3314,7 +3308,7 @@
         <v>7</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
     </row>
   </sheetData>

</xml_diff>